<commit_message>
Cap nhật project 16
</commit_message>
<xml_diff>
--- a/MosTrainer/Projects/Excel2019_P15/starter.xlsx
+++ b/MosTrainer/Projects/Excel2019_P15/starter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Excel cor\الكامل اكسيل 2019\Ex2019b\6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Việt Âu\MOS-EXCEL\EXCEL\Desktop du an\Excel2019_P15\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40919E50-D4A9-4AE4-A9B0-68A3B04DD77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30228C04-89B2-4441-B281-1B2B30B4FA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48" yWindow="72" windowWidth="22956" windowHeight="8496" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="El3ameed" sheetId="1" r:id="rId1"/>
@@ -458,7 +458,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$\ #,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -636,34 +636,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="44">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="4" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -672,101 +672,101 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="3" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="4" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="4" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="4"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="4" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,13 +856,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF6FAC46"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color rgb="FF6FAC46"/>
         </left>
@@ -872,6 +865,13 @@
         <top style="thin">
           <color rgb="FF6FAC46"/>
         </top>
+        <bottom style="thin">
+          <color rgb="FF6FAC46"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="thin">
           <color rgb="FF6FAC46"/>
         </bottom>
@@ -930,7 +930,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ar-EG"/>
+          <a:endParaRPr lang="vi-VN"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -956,6 +956,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-A547-4D40-BE28-9B82F9D1157C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -971,6 +976,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-A547-4D40-BE28-9B82F9D1157C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -986,6 +996,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-A547-4D40-BE28-9B82F9D1157C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -1001,6 +1016,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-A547-4D40-BE28-9B82F9D1157C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -1095,7 +1115,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ar-EG"/>
+          <a:endParaRPr lang="vi-VN"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1132,7 +1152,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="ar-EG"/>
+      <a:endParaRPr lang="vi-VN"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1206,7 +1226,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ar-EG"/>
+          <a:endParaRPr lang="vi-VN"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1354,8 +1374,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -1375,7 +1396,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ar-EG"/>
+            <a:endParaRPr lang="vi-VN"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1326513263"/>
@@ -1436,7 +1457,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="ar-EG"/>
+            <a:endParaRPr lang="vi-VN"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1326510767"/>
@@ -1487,7 +1508,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="ar-EG"/>
+      <a:endParaRPr lang="vi-VN"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2718,7 +2739,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8B4DB20-58A0-4901-873E-F653A77EF09E}" name="Table1" displayName="Table1" ref="A3:B7" totalsRowShown="0" headerRowBorderDxfId="3" tableBorderDxfId="4" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8B4DB20-58A0-4901-873E-F653A77EF09E}" name="Table1" displayName="Table1" ref="A3:B7" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="A3:B7" xr:uid="{C8B4DB20-58A0-4901-873E-F653A77EF09E}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{8B71D2AD-95C4-4F82-AD29-7B2E4F7980E6}" name="Program" dataDxfId="1"/>
@@ -3050,39 +3071,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.1640625" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
     <col min="4" max="4" width="56" customWidth="1"/>
-    <col min="5" max="5" width="115.83203125" customWidth="1"/>
+    <col min="5" max="5" width="115.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" customHeight="1">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-    </row>
-    <row r="2" spans="1:5" ht="16.5" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="B1" s="28"/>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-    </row>
-    <row r="3" spans="1:5" ht="16.5" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+    </row>
+    <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" customHeight="1">
+    <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -3090,7 +3111,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16.5" customHeight="1">
+    <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
@@ -3098,7 +3119,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" customHeight="1">
+    <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
@@ -3106,11 +3127,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" customHeight="1">
-      <c r="A7" s="35" t="s">
+    <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="36">
+      <c r="B7" s="22">
         <v>63</v>
       </c>
     </row>
@@ -3130,527 +3151,544 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I41"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.5" customWidth="1"/>
-    <col min="2" max="2" width="1.1640625" customWidth="1"/>
-    <col min="3" max="3" width="2.83203125" customWidth="1"/>
+    <col min="1" max="1" width="37.44140625" customWidth="1"/>
+    <col min="2" max="2" width="1.109375" customWidth="1"/>
+    <col min="3" max="3" width="2.77734375" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="3.1640625" customWidth="1"/>
+    <col min="6" max="6" width="3.109375" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" customHeight="1">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-    </row>
-    <row r="2" spans="1:9" ht="21" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+    </row>
+    <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-    </row>
-    <row r="3" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A3" s="41" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+    </row>
+    <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42" t="s">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="29" t="s">
+      <c r="B4" s="39"/>
+      <c r="C4" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="38" t="s">
+      <c r="D4" s="39"/>
+      <c r="E4" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="39"/>
-      <c r="H4" s="13" t="s">
+      <c r="G4" s="41"/>
+      <c r="H4" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="43" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A5" s="30" t="s">
+    <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="32" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="32"/>
+      <c r="D5" s="33"/>
       <c r="E5" s="9">
         <v>18</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="30">
         <v>2</v>
       </c>
-      <c r="G5" s="24"/>
-      <c r="H5" s="15">
+      <c r="G5" s="30"/>
+      <c r="H5" s="14">
         <v>3800</v>
       </c>
-      <c r="I5" s="16">
+      <c r="I5" s="15">
         <v>68400</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A6" s="30" t="s">
+    <row r="6" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="32" t="s">
+      <c r="B6" s="32"/>
+      <c r="C6" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="32"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="9">
         <v>0</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="30">
         <v>1</v>
       </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="15">
+      <c r="G6" s="30"/>
+      <c r="H6" s="14">
         <v>10000</v>
       </c>
-      <c r="I6" s="17" t="s">
+      <c r="I6" s="16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="32" t="s">
+      <c r="B7" s="32"/>
+      <c r="C7" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="32"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="9">
         <v>3</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="30">
         <v>2</v>
       </c>
-      <c r="G7" s="24"/>
-      <c r="H7" s="15">
+      <c r="G7" s="30"/>
+      <c r="H7" s="14">
         <v>4000</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="15">
         <v>12000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="32" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="32"/>
+      <c r="D8" s="33"/>
       <c r="E8" s="9">
         <v>15</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="30">
         <v>1</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="15">
+      <c r="G8" s="30"/>
+      <c r="H8" s="14">
         <v>3750</v>
       </c>
-      <c r="I8" s="16">
+      <c r="I8" s="15">
         <v>56250</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A9" s="30" t="s">
+    <row r="9" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="32" t="s">
+      <c r="B9" s="32"/>
+      <c r="C9" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="32"/>
+      <c r="D9" s="33"/>
       <c r="E9" s="9">
         <v>13</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="30">
         <v>3</v>
       </c>
-      <c r="G9" s="24"/>
-      <c r="H9" s="15">
+      <c r="G9" s="30"/>
+      <c r="H9" s="14">
         <v>8000</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="15">
         <v>104000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="30" t="s">
+    <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="32" t="s">
+      <c r="B10" s="32"/>
+      <c r="C10" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="32"/>
+      <c r="D10" s="33"/>
       <c r="E10" s="9">
         <v>12</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="30">
         <v>2</v>
       </c>
-      <c r="G10" s="24"/>
-      <c r="H10" s="15">
+      <c r="G10" s="30"/>
+      <c r="H10" s="14">
         <v>7500</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="15">
         <v>90000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A11" s="30" t="s">
+    <row r="11" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="32" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="32"/>
+      <c r="D11" s="33"/>
       <c r="E11" s="9">
         <v>3</v>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="30">
         <v>2</v>
       </c>
-      <c r="G11" s="24"/>
-      <c r="H11" s="15">
+      <c r="G11" s="30"/>
+      <c r="H11" s="14">
         <v>4300</v>
       </c>
-      <c r="I11" s="16">
+      <c r="I11" s="15">
         <v>12900</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A12" s="30" t="s">
+    <row r="12" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="31"/>
-      <c r="C12" s="32" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="32"/>
+      <c r="D12" s="33"/>
       <c r="E12" s="9">
         <v>12</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="30">
         <v>2</v>
       </c>
-      <c r="G12" s="24"/>
-      <c r="H12" s="15">
+      <c r="G12" s="30"/>
+      <c r="H12" s="14">
         <v>3000</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="15">
         <v>36000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A13" s="30" t="s">
+    <row r="13" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="32" t="s">
+      <c r="B13" s="32"/>
+      <c r="C13" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="32"/>
+      <c r="D13" s="33"/>
       <c r="E13" s="9">
         <v>8</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="30">
         <v>2</v>
       </c>
-      <c r="G13" s="24"/>
-      <c r="H13" s="15">
+      <c r="G13" s="30"/>
+      <c r="H13" s="14">
         <v>4500</v>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="15">
         <v>36000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A14" s="30" t="s">
+    <row r="14" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="32" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="32"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="9">
         <v>11</v>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="30">
         <v>1</v>
       </c>
-      <c r="G14" s="24"/>
-      <c r="H14" s="15">
+      <c r="G14" s="30"/>
+      <c r="H14" s="14">
         <v>7500</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="15">
         <v>82500</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A15" s="30" t="s">
+    <row r="15" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="32" t="s">
+      <c r="B15" s="32"/>
+      <c r="C15" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="32"/>
+      <c r="D15" s="33"/>
       <c r="E15" s="9">
         <v>8</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="30">
         <v>2</v>
       </c>
-      <c r="G15" s="24"/>
-      <c r="H15" s="15">
+      <c r="G15" s="30"/>
+      <c r="H15" s="14">
         <v>3200</v>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="15">
         <v>25600</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A16" s="30" t="s">
+    <row r="16" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="32" t="s">
+      <c r="B16" s="32"/>
+      <c r="C16" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="32"/>
+      <c r="D16" s="33"/>
       <c r="E16" s="9">
         <v>4</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="30">
         <v>1</v>
       </c>
-      <c r="G16" s="24"/>
-      <c r="H16" s="15">
+      <c r="G16" s="30"/>
+      <c r="H16" s="14">
         <v>5000</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="15">
         <v>20000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="32" t="s">
+      <c r="B17" s="32"/>
+      <c r="C17" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="32"/>
+      <c r="D17" s="33"/>
       <c r="E17" s="9">
         <v>7</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="30">
         <v>1</v>
       </c>
-      <c r="G17" s="24"/>
-      <c r="H17" s="15">
+      <c r="G17" s="30"/>
+      <c r="H17" s="14">
         <v>6500</v>
       </c>
-      <c r="I17" s="16">
+      <c r="I17" s="15">
         <v>45500</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A18" s="30" t="s">
+    <row r="18" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="32" t="s">
+      <c r="B18" s="32"/>
+      <c r="C18" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="32"/>
+      <c r="D18" s="33"/>
       <c r="E18" s="9">
         <v>9</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="30">
         <v>1</v>
       </c>
-      <c r="G18" s="24"/>
-      <c r="H18" s="15">
+      <c r="G18" s="30"/>
+      <c r="H18" s="14">
         <v>3500</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="15">
         <v>31500</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="30" t="s">
+    <row r="19" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="32" t="s">
+      <c r="B19" s="32"/>
+      <c r="C19" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="32"/>
+      <c r="D19" s="33"/>
       <c r="E19" s="9">
         <v>2</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="30">
         <v>2</v>
       </c>
-      <c r="G19" s="24"/>
-      <c r="H19" s="15">
+      <c r="G19" s="30"/>
+      <c r="H19" s="14">
         <v>2000</v>
       </c>
-      <c r="I19" s="16">
+      <c r="I19" s="15">
         <v>14000</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="32" t="s">
+      <c r="B20" s="32"/>
+      <c r="C20" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="32"/>
+      <c r="D20" s="33"/>
       <c r="E20" s="9">
         <v>12</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="30">
         <v>3</v>
       </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="15">
+      <c r="G20" s="30"/>
+      <c r="H20" s="14">
         <v>6450</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="15">
         <v>77400</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A21" s="30" t="s">
+    <row r="21" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="32" t="s">
+      <c r="B21" s="32"/>
+      <c r="C21" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="32"/>
+      <c r="D21" s="33"/>
       <c r="E21" s="9">
         <v>5</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="30">
         <v>1</v>
       </c>
-      <c r="G21" s="24"/>
-      <c r="H21" s="15">
+      <c r="G21" s="30"/>
+      <c r="H21" s="14">
         <v>4250</v>
       </c>
-      <c r="I21" s="16">
+      <c r="I21" s="15">
         <v>21250</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="31"/>
-      <c r="C22" s="32" t="s">
+      <c r="B22" s="32"/>
+      <c r="C22" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="32"/>
+      <c r="D22" s="33"/>
       <c r="E22" s="9">
         <v>3</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="30">
         <v>1</v>
       </c>
-      <c r="G22" s="24"/>
-      <c r="H22" s="15">
+      <c r="G22" s="30"/>
+      <c r="H22" s="14">
         <v>3000</v>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="15">
         <v>9000</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="33" customHeight="1"/>
-    <row r="24" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="25" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="26" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="27" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="28" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="29" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="30" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="31" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="32" spans="1:9" ht="16.5" customHeight="1"/>
-    <row r="33" ht="16.5" customHeight="1"/>
-    <row r="34" ht="16.5" customHeight="1"/>
-    <row r="35" ht="16.5" customHeight="1"/>
-    <row r="36" ht="16.5" customHeight="1"/>
-    <row r="37" ht="16.5" customHeight="1"/>
-    <row r="38" ht="16.5" customHeight="1"/>
-    <row r="39" ht="16.5" customHeight="1"/>
-    <row r="40" ht="16.5" customHeight="1"/>
-    <row r="41" ht="16.5" customHeight="1"/>
+    <row r="23" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="A22:B22"/>
@@ -3659,41 +3697,24 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="C20:D20"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3702,13 +3723,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F38"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" customHeight="1">
+    <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -3724,11 +3745,11 @@
       <c r="E1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="16.5" customHeight="1">
+    <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -3741,14 +3762,14 @@
       <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="18">
+      <c r="E2" s="17">
         <v>3800</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="15">
         <v>57000</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="16.5" customHeight="1">
+    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -3761,15 +3782,15 @@
       <c r="D3" s="12">
         <v>1</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>10000</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="15">
         <v>130000</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A4" s="43" t="s">
+    <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>41</v>
       </c>
       <c r="B4" s="8" t="s">
@@ -3781,14 +3802,14 @@
       <c r="D4" s="12">
         <v>2</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="17">
         <v>4000</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="15">
         <v>16000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="16.5" customHeight="1">
+    <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -3801,14 +3822,14 @@
       <c r="D5" s="12">
         <v>1</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <v>3750</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="15">
         <v>41250</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="16.5" customHeight="1">
+    <row r="6" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -3821,14 +3842,14 @@
       <c r="D6" s="12">
         <v>3</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>8000</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="15">
         <v>104000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="16.5" customHeight="1">
+    <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -3841,14 +3862,14 @@
       <c r="D7" s="12">
         <v>1</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>7500</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="15">
         <v>105000</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="16.5" customHeight="1">
+    <row r="8" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -3861,14 +3882,14 @@
       <c r="D8" s="12">
         <v>2</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>4300</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="15">
         <v>17200</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="16.5" customHeight="1">
+    <row r="9" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
@@ -3881,14 +3902,14 @@
       <c r="D9" s="12">
         <v>2</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>3000</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="15">
         <v>24000</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="16.5" customHeight="1">
+    <row r="10" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -3901,14 +3922,14 @@
       <c r="D10" s="12">
         <v>3</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <v>4500</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="15">
         <v>22500</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="16.5" customHeight="1">
+    <row r="11" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
@@ -3921,14 +3942,14 @@
       <c r="D11" s="12">
         <v>1</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>7500</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="15">
         <v>60000</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="16.5" customHeight="1">
+    <row r="12" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -3941,14 +3962,14 @@
       <c r="D12" s="12">
         <v>2</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>3200</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="15">
         <v>25600</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="16.5" customHeight="1">
+    <row r="13" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
@@ -3961,14 +3982,14 @@
       <c r="D13" s="12">
         <v>1</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>5000</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="15">
         <v>65000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="16.5" customHeight="1">
+    <row r="14" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -3981,14 +4002,14 @@
       <c r="D14" s="12">
         <v>1</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>6500</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="15">
         <v>65000</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="16.5" customHeight="1">
+    <row r="15" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>23</v>
       </c>
@@ -4001,14 +4022,14 @@
       <c r="D15" s="12">
         <v>1</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>3500</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="15">
         <v>24500</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="16.5" customHeight="1">
+    <row r="16" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>24</v>
       </c>
@@ -4021,14 +4042,14 @@
       <c r="D16" s="12">
         <v>2</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>2000</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="15">
         <v>22000</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="16.5" customHeight="1">
+    <row r="17" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
@@ -4041,14 +4062,14 @@
       <c r="D17" s="12">
         <v>2</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <v>6450</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="15">
         <v>58050</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="16.5" customHeight="1">
+    <row r="18" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>26</v>
       </c>
@@ -4061,14 +4082,14 @@
       <c r="D18" s="12">
         <v>2</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <v>4250</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="15">
         <v>51000</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="16.5" customHeight="1">
+    <row r="19" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
@@ -4081,32 +4102,32 @@
       <c r="D19" s="12">
         <v>1</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <v>3000</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="15">
         <v>15000</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="33" customHeight="1"/>
-    <row r="21" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="22" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="23" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="24" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="25" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="26" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="27" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="28" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="29" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="30" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="31" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="32" spans="1:6" ht="16.5" customHeight="1"/>
-    <row r="33" ht="16.5" customHeight="1"/>
-    <row r="34" ht="16.5" customHeight="1"/>
-    <row r="35" ht="16.5" customHeight="1"/>
-    <row r="36" ht="16.5" customHeight="1"/>
-    <row r="37" ht="16.5" customHeight="1"/>
-    <row r="38" ht="16.5" customHeight="1"/>
+    <row r="20" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4115,75 +4136,75 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.5" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" customWidth="1"/>
     <col min="3" max="3" width="58" customWidth="1"/>
-    <col min="4" max="4" width="2.5" customWidth="1"/>
+    <col min="4" max="4" width="2.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" customHeight="1">
+    <row r="1" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-    </row>
-    <row r="2" spans="1:4" ht="16.5" customHeight="1">
+      <c r="B1" s="18"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+    </row>
+    <row r="2" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-    </row>
-    <row r="3" spans="1:4" ht="16.5" customHeight="1">
+      <c r="B2" s="18"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-    </row>
-    <row r="4" spans="1:4" ht="16.5" customHeight="1">
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="19">
         <v>282400</v>
       </c>
-      <c r="C4" s="20"/>
-    </row>
-    <row r="5" spans="1:4" ht="16.5" customHeight="1">
+      <c r="C4" s="19"/>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="19">
         <v>103100</v>
       </c>
-      <c r="C5" s="20"/>
-    </row>
-    <row r="6" spans="1:4" ht="16.5" customHeight="1">
+      <c r="C5" s="19"/>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="19">
         <v>172800</v>
       </c>
-      <c r="C6" s="20"/>
-    </row>
-    <row r="7" spans="1:4" ht="16.5" customHeight="1">
+      <c r="C6" s="19"/>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="19">
         <v>183000</v>
       </c>
-      <c r="C7" s="20"/>
+      <c r="C7" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>